<commit_message>
chore: rerun DiD analyses with 100 bootstrap reps
</commit_message>
<xml_diff>
--- a/analysis/econometrics_outputs/contdid/Graficos/contracts/contdid_cosine_nearest_continuous.xlsx
+++ b/analysis/econometrics_outputs/contdid/Graficos/contracts/contdid_cosine_nearest_continuous.xlsx
@@ -407,7 +407,7 @@
     <col min="5" max="5" width="13.67625" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="11.31875" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="13.67625" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="13.67625" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="12.4975" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="12.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="5.425" hidden="0" customWidth="1"/>
     <col min="11" max="11" width="3.71" hidden="0" customWidth="1"/>
@@ -515,13 +515,13 @@
         <v>1542.0906</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>1831.3548</v>
+        <v>1685.8873</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>-35097.1522</v>
+        <v>-2971.6862</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>38181.3334</v>
+        <v>6055.8675</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>10</v>
@@ -543,13 +543,13 @@
         <v>-628.5425</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>3395.4634</v>
+        <v>2954.5597</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>-68560.3315</v>
+        <v>-8539.0495</v>
       </c>
       <c r="H7" s="1" t="n">
-        <v>67303.2465</v>
+        <v>7281.9646</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>10</v>
@@ -571,13 +571,13 @@
         <v>2244.3985</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>1548.3213</v>
+        <v>1204.07</v>
       </c>
       <c r="G8" s="1" t="n">
-        <v>-28732.296</v>
+        <v>-979.3658</v>
       </c>
       <c r="H8" s="1" t="n">
-        <v>33221.0929</v>
+        <v>5468.1627</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>10</v>
@@ -599,16 +599,16 @@
         <v>-10766.9938</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>3498.9735</v>
+        <v>3857.3169</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>-80769.6713</v>
+        <v>-21094.5335</v>
       </c>
       <c r="H9" s="1" t="n">
-        <v>59235.6837</v>
+        <v>-439.4541</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>11</v>
@@ -627,13 +627,13 @@
         <v>1431.8624</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>1655.7112</v>
+        <v>2423.2172</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>-31693.3442</v>
+        <v>-5056.0338</v>
       </c>
       <c r="H10" s="1" t="n">
-        <v>34557.069</v>
+        <v>7919.7586</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>10</v>
@@ -655,13 +655,13 @@
         <v>7903.8528</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>3886.1366</v>
+        <v>4251.8997</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>-69844.6546</v>
+        <v>-3480.1387</v>
       </c>
       <c r="H11" s="1" t="n">
-        <v>85652.3603</v>
+        <v>19287.8443</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>10</v>
@@ -683,13 +683,13 @@
         <v>6519.8733</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>1356.9479</v>
+        <v>2887.4986</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>-20628.084</v>
+        <v>-1211.0852</v>
       </c>
       <c r="H12" s="1" t="n">
-        <v>33667.8307</v>
+        <v>14250.8318</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>10</v>
@@ -711,13 +711,13 @@
         <v>-13932.1192</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>7157.2551</v>
+        <v>9366.0591</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>-157124.6933</v>
+        <v>-39008.7075</v>
       </c>
       <c r="H13" s="1" t="n">
-        <v>129260.4549</v>
+        <v>11144.4691</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>10</v>
@@ -739,13 +739,13 @@
         <v>-1302.7618</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>3019.9888</v>
+        <v>2173.3957</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>-61722.5692</v>
+        <v>-7121.7885</v>
       </c>
       <c r="H14" s="1" t="n">
-        <v>59117.0455</v>
+        <v>4516.2649</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>10</v>
@@ -767,13 +767,13 @@
         <v>-6685.5233</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>1029.2759</v>
+        <v>5349.7086</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>-27277.869</v>
+        <v>-21008.777</v>
       </c>
       <c r="H15" s="1" t="n">
-        <v>13906.8224</v>
+        <v>7637.7304</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>10</v>
@@ -795,13 +795,13 @@
         <v>3385.0498</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>289.3097</v>
+        <v>1808.7259</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>-2403.0632</v>
+        <v>-1457.6139</v>
       </c>
       <c r="H16" s="1" t="n">
-        <v>9173.1628</v>
+        <v>8227.7135</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>10</v>
@@ -823,13 +823,13 @@
         <v>4736.8659</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>2125.6742</v>
+        <v>2103.1607</v>
       </c>
       <c r="G17" s="1" t="n">
-        <v>-37790.7163</v>
+        <v>-894.1146</v>
       </c>
       <c r="H17" s="1" t="n">
-        <v>47264.4482</v>
+        <v>10367.8464</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>10</v>
@@ -851,16 +851,16 @@
         <v>7691.8381</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>376.6856</v>
+        <v>7432.8506</v>
       </c>
       <c r="G18" s="1" t="n">
-        <v>155.627</v>
+        <v>-12208.7981</v>
       </c>
       <c r="H18" s="1" t="n">
-        <v>15228.0491</v>
+        <v>27592.4743</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>11</v>
@@ -879,13 +879,13 @@
         <v>-2044.5024</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>1046.7211</v>
+        <v>2432.6512</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>-22985.8663</v>
+        <v>-8557.6572</v>
       </c>
       <c r="H19" s="1" t="n">
-        <v>18896.8615</v>
+        <v>4468.6524</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>10</v>
@@ -907,13 +907,13 @@
         <v>3980.763</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>1911.1541</v>
+        <v>2726.6823</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>-34254.9949</v>
+        <v>-3319.6277</v>
       </c>
       <c r="H20" s="1" t="n">
-        <v>42216.5209</v>
+        <v>11281.1536</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>10</v>
@@ -935,13 +935,13 @@
         <v>-6660.7928</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>4168.3375</v>
+        <v>4092.041</v>
       </c>
       <c r="G21" s="1" t="n">
-        <v>-90055.1895</v>
+        <v>-17616.7804</v>
       </c>
       <c r="H21" s="1" t="n">
-        <v>76733.6039</v>
+        <v>4295.1949</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>10</v>
@@ -963,13 +963,13 @@
         <v>6084.3306</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>2163.4824</v>
+        <v>2498.6385</v>
       </c>
       <c r="G22" s="1" t="n">
-        <v>-37199.6665</v>
+        <v>-605.4979</v>
       </c>
       <c r="H22" s="1" t="n">
-        <v>49368.3278</v>
+        <v>12774.1591</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>10</v>
@@ -991,13 +991,13 @@
         <v>8178.6453</v>
       </c>
       <c r="F23" s="1" t="n">
-        <v>894.2479</v>
+        <v>4279.8331</v>
       </c>
       <c r="G23" s="1" t="n">
-        <v>-9712.2449</v>
+        <v>-3280.1348</v>
       </c>
       <c r="H23" s="1" t="n">
-        <v>26069.5355</v>
+        <v>19637.4254</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>10</v>
@@ -1019,16 +1019,16 @@
         <v>4263.6724</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>96.7497</v>
+        <v>1852.2821</v>
       </c>
       <c r="G24" s="1" t="n">
-        <v>2328.0364</v>
+        <v>-695.6083</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>6199.3084</v>
+        <v>9222.9531</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>11</v>
@@ -1047,16 +1047,16 @@
         <v>-9914.2877</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>158.2787</v>
+        <v>6977.7049</v>
       </c>
       <c r="G25" s="1" t="n">
-        <v>-13080.9116</v>
+        <v>-28596.3216</v>
       </c>
       <c r="H25" s="1" t="n">
-        <v>-6747.6638</v>
+        <v>8767.7462</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J25" s="1" t="s">
         <v>13</v>
@@ -1075,13 +1075,13 @@
         <v>-7773.7163</v>
       </c>
       <c r="F26" s="1" t="n">
-        <v>2088.7795</v>
+        <v>4056.8783</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>-49563.1611</v>
+        <v>-18635.5595</v>
       </c>
       <c r="H26" s="1" t="n">
-        <v>34015.7285</v>
+        <v>3088.1269</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>10</v>
@@ -1103,13 +1103,13 @@
         <v>-8411.9515</v>
       </c>
       <c r="F27" s="1" t="n">
-        <v>1236.7448</v>
+        <v>5626.9196</v>
       </c>
       <c r="G27" s="1" t="n">
-        <v>-33155.0507</v>
+        <v>-23477.407</v>
       </c>
       <c r="H27" s="1" t="n">
-        <v>16331.1478</v>
+        <v>6653.5041</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>10</v>
@@ -1131,13 +1131,13 @@
         <v>-8816.5242</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>7093.3105</v>
+        <v>6993.657</v>
       </c>
       <c r="G28" s="1" t="n">
-        <v>-150729.7814</v>
+        <v>-27541.268</v>
       </c>
       <c r="H28" s="1" t="n">
-        <v>133096.7331</v>
+        <v>9908.2197</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>10</v>
@@ -1159,13 +1159,13 @@
         <v>-8148.4441</v>
       </c>
       <c r="F29" s="1" t="n">
-        <v>4558.2499</v>
+        <v>6703.6867</v>
       </c>
       <c r="G29" s="1" t="n">
-        <v>-99343.6759</v>
+        <v>-26096.8245</v>
       </c>
       <c r="H29" s="1" t="n">
-        <v>83046.7877</v>
+        <v>9799.9363</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>10</v>
@@ -1187,13 +1187,13 @@
         <v>-242.7521</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>511.7768</v>
+        <v>1568.5494</v>
       </c>
       <c r="G30" s="1" t="n">
-        <v>-10481.6833</v>
+        <v>-4442.3699</v>
       </c>
       <c r="H30" s="1" t="n">
-        <v>9996.1791</v>
+        <v>3956.8656</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>10</v>
@@ -1215,16 +1215,16 @@
         <v>-5509.5948</v>
       </c>
       <c r="F31" s="1" t="n">
-        <v>659.7116</v>
+        <v>1545.1042</v>
       </c>
       <c r="G31" s="1" t="n">
-        <v>-18708.2022</v>
+        <v>-9646.4406</v>
       </c>
       <c r="H31" s="1" t="n">
-        <v>7689.0126</v>
+        <v>-1372.749</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J31" s="1" t="s">
         <v>13</v>
@@ -1243,16 +1243,16 @@
         <v>-5314.0465</v>
       </c>
       <c r="F32" s="1" t="n">
-        <v>1203.1229</v>
+        <v>1500.7979</v>
       </c>
       <c r="G32" s="1" t="n">
-        <v>-29384.4837</v>
+        <v>-9332.2671</v>
       </c>
       <c r="H32" s="1" t="n">
-        <v>18756.3907</v>
+        <v>-1295.8258</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>13</v>
@@ -1271,16 +1271,16 @@
         <v>-10765.3347</v>
       </c>
       <c r="F33" s="1" t="n">
-        <v>2641.3699</v>
+        <v>3609.0491</v>
       </c>
       <c r="G33" s="1" t="n">
-        <v>-63610.2517</v>
+        <v>-20428.1648</v>
       </c>
       <c r="H33" s="1" t="n">
-        <v>42079.5824</v>
+        <v>-1102.5045</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>13</v>
@@ -1299,13 +1299,13 @@
         <v>-5228.2762</v>
       </c>
       <c r="F34" s="1" t="n">
-        <v>745.2507</v>
+        <v>2183.0259</v>
       </c>
       <c r="G34" s="1" t="n">
-        <v>-20138.2332</v>
+        <v>-11073.0867</v>
       </c>
       <c r="H34" s="1" t="n">
-        <v>9681.6808</v>
+        <v>616.5342</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>10</v>
@@ -1327,13 +1327,13 @@
         <v>-58.1705</v>
       </c>
       <c r="F35" s="1" t="n">
-        <v>976.8111</v>
+        <v>1220.6379</v>
       </c>
       <c r="G35" s="1" t="n">
-        <v>-19600.8705</v>
+        <v>-3326.2935</v>
       </c>
       <c r="H35" s="1" t="n">
-        <v>19484.5294</v>
+        <v>3209.9524</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>10</v>
@@ -1355,13 +1355,13 @@
         <v>2036.0752</v>
       </c>
       <c r="F36" s="1" t="n">
-        <v>535.4155</v>
+        <v>1114.5654</v>
       </c>
       <c r="G36" s="1" t="n">
-        <v>-8675.7854</v>
+        <v>-948.0506</v>
       </c>
       <c r="H36" s="1" t="n">
-        <v>12747.9357</v>
+        <v>5020.201</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>10</v>
@@ -1383,13 +1383,13 @@
         <v>-4794.6963</v>
       </c>
       <c r="F37" s="1" t="n">
-        <v>3010.8513</v>
+        <v>3518.9256</v>
       </c>
       <c r="G37" s="1" t="n">
-        <v>-65031.6929</v>
+        <v>-14216.2307</v>
       </c>
       <c r="H37" s="1" t="n">
-        <v>55442.3002</v>
+        <v>4626.8381</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>10</v>
@@ -1411,13 +1411,13 @@
         <v>-4090.1501</v>
       </c>
       <c r="F38" s="1" t="n">
-        <v>1439.8786</v>
+        <v>2026.6191</v>
       </c>
       <c r="G38" s="1" t="n">
-        <v>-32897.2722</v>
+        <v>-9516.1989</v>
       </c>
       <c r="H38" s="1" t="n">
-        <v>24716.972</v>
+        <v>1335.8986</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>10</v>
@@ -1439,13 +1439,13 @@
         <v>-8253.5303</v>
       </c>
       <c r="F39" s="1" t="n">
-        <v>2201.5554</v>
+        <v>5577.1843</v>
       </c>
       <c r="G39" s="1" t="n">
-        <v>-52299.2411</v>
+        <v>-23185.8251</v>
       </c>
       <c r="H39" s="1" t="n">
-        <v>35792.1805</v>
+        <v>6678.7645</v>
       </c>
       <c r="I39" s="1" t="s">
         <v>10</v>
@@ -1467,13 +1467,13 @@
         <v>-5576.5705</v>
       </c>
       <c r="F40" s="1" t="n">
-        <v>1335.0777</v>
+        <v>5458.7417</v>
       </c>
       <c r="G40" s="1" t="n">
-        <v>-32286.9805</v>
+        <v>-20191.7481</v>
       </c>
       <c r="H40" s="1" t="n">
-        <v>21133.8395</v>
+        <v>9038.6071</v>
       </c>
       <c r="I40" s="1" t="s">
         <v>10</v>
@@ -1495,13 +1495,13 @@
         <v>-1879.3838</v>
       </c>
       <c r="F41" s="1" t="n">
-        <v>1657.3594</v>
+        <v>2904.5514</v>
       </c>
       <c r="G41" s="1" t="n">
-        <v>-35037.5646</v>
+        <v>-9655.9994</v>
       </c>
       <c r="H41" s="1" t="n">
-        <v>31278.7969</v>
+        <v>5897.2317</v>
       </c>
       <c r="I41" s="1" t="s">
         <v>10</v>
@@ -1523,13 +1523,13 @@
         <v>-202.2197</v>
       </c>
       <c r="F42" s="1" t="n">
-        <v>273.2765</v>
+        <v>1041.9297</v>
       </c>
       <c r="G42" s="1" t="n">
-        <v>-5669.5619</v>
+        <v>-2991.8713</v>
       </c>
       <c r="H42" s="1" t="n">
-        <v>5265.1226</v>
+        <v>2587.432</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>10</v>
@@ -1551,13 +1551,13 @@
         <v>-424.7903</v>
       </c>
       <c r="F43" s="1" t="n">
-        <v>553.05</v>
+        <v>812.1043</v>
       </c>
       <c r="G43" s="1" t="n">
-        <v>-11489.4591</v>
+        <v>-2599.1098</v>
       </c>
       <c r="H43" s="1" t="n">
-        <v>10639.8785</v>
+        <v>1749.5292</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>10</v>
@@ -1579,16 +1579,16 @@
         <v>-4688.4677</v>
       </c>
       <c r="F44" s="1" t="n">
-        <v>1062.272</v>
+        <v>1449.9873</v>
       </c>
       <c r="G44" s="1" t="n">
-        <v>-25940.9526</v>
+        <v>-8570.6486</v>
       </c>
       <c r="H44" s="1" t="n">
-        <v>16564.0172</v>
+        <v>-806.2868</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J44" s="1" t="s">
         <v>13</v>
@@ -1607,13 +1607,13 @@
         <v>-6592.6021</v>
       </c>
       <c r="F45" s="1" t="n">
-        <v>3528.8525</v>
+        <v>2515.5887</v>
       </c>
       <c r="G45" s="1" t="n">
-        <v>-77193.0568</v>
+        <v>-13327.813</v>
       </c>
       <c r="H45" s="1" t="n">
-        <v>64007.8525</v>
+        <v>142.6088</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>10</v>
@@ -1635,13 +1635,13 @@
         <v>-114.3333</v>
       </c>
       <c r="F46" s="1" t="n">
-        <v>321.0827</v>
+        <v>1276.7066</v>
       </c>
       <c r="G46" s="1" t="n">
-        <v>-6538.1171</v>
+        <v>-3532.5741</v>
       </c>
       <c r="H46" s="1" t="n">
-        <v>6309.4504</v>
+        <v>3303.9074</v>
       </c>
       <c r="I46" s="1" t="s">
         <v>10</v>
@@ -1663,13 +1663,13 @@
         <v>95.0024</v>
       </c>
       <c r="F47" s="1" t="n">
-        <v>1566.6744</v>
+        <v>1993.4389</v>
       </c>
       <c r="G47" s="1" t="n">
-        <v>-31248.8775</v>
+        <v>-5242.2099</v>
       </c>
       <c r="H47" s="1" t="n">
-        <v>31438.8823</v>
+        <v>5432.2147</v>
       </c>
       <c r="I47" s="1" t="s">
         <v>10</v>
@@ -1691,13 +1691,13 @@
         <v>5384.0509</v>
       </c>
       <c r="F48" s="1" t="n">
-        <v>513.2121</v>
+        <v>2215.1974</v>
       </c>
       <c r="G48" s="1" t="n">
-        <v>-4883.5945</v>
+        <v>-546.8953</v>
       </c>
       <c r="H48" s="1" t="n">
-        <v>15651.6962</v>
+        <v>11314.9971</v>
       </c>
       <c r="I48" s="1" t="s">
         <v>10</v>
@@ -1719,13 +1719,13 @@
         <v>-2388.2933</v>
       </c>
       <c r="F49" s="1" t="n">
-        <v>1331.4213</v>
+        <v>2558.2099</v>
       </c>
       <c r="G49" s="1" t="n">
-        <v>-29025.5493</v>
+        <v>-9237.6176</v>
       </c>
       <c r="H49" s="1" t="n">
-        <v>24248.9626</v>
+        <v>4461.0309</v>
       </c>
       <c r="I49" s="1" t="s">
         <v>10</v>
@@ -1747,13 +1747,13 @@
         <v>-2340.3333</v>
       </c>
       <c r="F50" s="1" t="n">
-        <v>807.3293</v>
+        <v>1936.0112</v>
       </c>
       <c r="G50" s="1" t="n">
-        <v>-18492.2747</v>
+        <v>-7523.7893</v>
       </c>
       <c r="H50" s="1" t="n">
-        <v>13811.6081</v>
+        <v>2843.1227</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>10</v>
@@ -1775,13 +1775,13 @@
         <v>-6424.4262</v>
       </c>
       <c r="F51" s="1" t="n">
-        <v>6082.1046</v>
+        <v>5580.328</v>
       </c>
       <c r="G51" s="1" t="n">
-        <v>-128106.8592</v>
+        <v>-21365.1378</v>
       </c>
       <c r="H51" s="1" t="n">
-        <v>115258.0068</v>
+        <v>8516.2854</v>
       </c>
       <c r="I51" s="1" t="s">
         <v>10</v>
@@ -1803,13 +1803,13 @@
         <v>-7500.7329</v>
       </c>
       <c r="F52" s="1" t="n">
-        <v>6963.2285</v>
+        <v>7095.6744</v>
       </c>
       <c r="G52" s="1" t="n">
-        <v>-146811.4872</v>
+        <v>-26498.6171</v>
       </c>
       <c r="H52" s="1" t="n">
-        <v>131810.0214</v>
+        <v>11497.1513</v>
       </c>
       <c r="I52" s="1" t="s">
         <v>10</v>
@@ -1831,13 +1831,13 @@
         <v>-3386.1301</v>
       </c>
       <c r="F53" s="1" t="n">
-        <v>4776.9987</v>
+        <v>5121.526</v>
       </c>
       <c r="G53" s="1" t="n">
-        <v>-98957.7883</v>
+        <v>-17098.4499</v>
       </c>
       <c r="H53" s="1" t="n">
-        <v>92185.5282</v>
+        <v>10326.1898</v>
       </c>
       <c r="I53" s="1" t="s">
         <v>10</v>
@@ -1859,13 +1859,13 @@
         <v>1094.4829</v>
       </c>
       <c r="F54" s="1" t="n">
-        <v>299.3326</v>
+        <v>1093.3271</v>
       </c>
       <c r="G54" s="1" t="n">
-        <v>-4894.1547</v>
+        <v>-1832.7795</v>
       </c>
       <c r="H54" s="1" t="n">
-        <v>7083.1204</v>
+        <v>4021.7453</v>
       </c>
       <c r="I54" s="1" t="s">
         <v>10</v>
@@ -1887,13 +1887,13 @@
         <v>3729.6699</v>
       </c>
       <c r="F55" s="1" t="n">
-        <v>2083.8689</v>
+        <v>1673.0288</v>
       </c>
       <c r="G55" s="1" t="n">
-        <v>-37961.5302</v>
+        <v>-749.6799</v>
       </c>
       <c r="H55" s="1" t="n">
-        <v>45420.87</v>
+        <v>8209.0197</v>
       </c>
       <c r="I55" s="1" t="s">
         <v>10</v>
@@ -1915,13 +1915,13 @@
         <v>213.8525</v>
       </c>
       <c r="F56" s="1" t="n">
-        <v>1213.3929</v>
+        <v>1448.6422</v>
       </c>
       <c r="G56" s="1" t="n">
-        <v>-24062.0531</v>
+        <v>-3664.7268</v>
       </c>
       <c r="H56" s="1" t="n">
-        <v>24489.7581</v>
+        <v>4092.4318</v>
       </c>
       <c r="I56" s="1" t="s">
         <v>10</v>
@@ -1943,13 +1943,13 @@
         <v>-5130.8868</v>
       </c>
       <c r="F57" s="1" t="n">
-        <v>900.9522</v>
+        <v>2100.9569</v>
       </c>
       <c r="G57" s="1" t="n">
-        <v>-23155.9074</v>
+        <v>-10755.9669</v>
       </c>
       <c r="H57" s="1" t="n">
-        <v>12894.1337</v>
+        <v>494.1932</v>
       </c>
       <c r="I57" s="1" t="s">
         <v>10</v>
@@ -1971,13 +1971,13 @@
         <v>-2165.6217</v>
       </c>
       <c r="F58" s="1" t="n">
-        <v>673.9657</v>
+        <v>1985.8318</v>
       </c>
       <c r="G58" s="1" t="n">
-        <v>-15649.4053</v>
+        <v>-7482.4669</v>
       </c>
       <c r="H58" s="1" t="n">
-        <v>11318.162</v>
+        <v>3151.2235</v>
       </c>
       <c r="I58" s="1" t="s">
         <v>10</v>
@@ -1999,13 +1999,13 @@
         <v>1321.8799</v>
       </c>
       <c r="F59" s="1" t="n">
-        <v>1173.524</v>
+        <v>2301.296</v>
       </c>
       <c r="G59" s="1" t="n">
-        <v>-22156.3831</v>
+        <v>-4839.5858</v>
       </c>
       <c r="H59" s="1" t="n">
-        <v>24800.1428</v>
+        <v>7483.3455</v>
       </c>
       <c r="I59" s="1" t="s">
         <v>10</v>
@@ -2027,13 +2027,13 @@
         <v>6092.1673</v>
       </c>
       <c r="F60" s="1" t="n">
-        <v>2200.7477</v>
+        <v>2404.5349</v>
       </c>
       <c r="G60" s="1" t="n">
-        <v>-37937.3842</v>
+        <v>-345.7093</v>
       </c>
       <c r="H60" s="1" t="n">
-        <v>50121.7188</v>
+        <v>12530.0439</v>
       </c>
       <c r="I60" s="1" t="s">
         <v>10</v>
@@ -2055,13 +2055,13 @@
         <v>-4232.1105</v>
       </c>
       <c r="F61" s="1" t="n">
-        <v>397.185</v>
+        <v>3083.9383</v>
       </c>
       <c r="G61" s="1" t="n">
-        <v>-12178.445</v>
+        <v>-12489.0145</v>
       </c>
       <c r="H61" s="1" t="n">
-        <v>3714.224</v>
+        <v>4024.7935</v>
       </c>
       <c r="I61" s="1" t="s">
         <v>10</v>
@@ -2083,13 +2083,13 @@
         <v>-4400.4057</v>
       </c>
       <c r="F62" s="1" t="n">
-        <v>669.6964</v>
+        <v>2257.7489</v>
       </c>
       <c r="G62" s="1" t="n">
-        <v>-17798.7751</v>
+        <v>-10445.2789</v>
       </c>
       <c r="H62" s="1" t="n">
-        <v>8997.9637</v>
+        <v>1644.4676</v>
       </c>
       <c r="I62" s="1" t="s">
         <v>10</v>
@@ -2111,13 +2111,13 @@
         <v>-2128.6234</v>
       </c>
       <c r="F63" s="1" t="n">
-        <v>2378.7624</v>
+        <v>3101.5839</v>
       </c>
       <c r="G63" s="1" t="n">
-        <v>-49719.6484</v>
+        <v>-10432.7716</v>
       </c>
       <c r="H63" s="1" t="n">
-        <v>45462.4015</v>
+        <v>6175.5248</v>
       </c>
       <c r="I63" s="1" t="s">
         <v>10</v>
@@ -2139,13 +2139,13 @@
         <v>-5858.881</v>
       </c>
       <c r="F64" s="1" t="n">
-        <v>2109.6589</v>
+        <v>5891.2859</v>
       </c>
       <c r="G64" s="1" t="n">
-        <v>-48066.0518</v>
+        <v>-21632.148</v>
       </c>
       <c r="H64" s="1" t="n">
-        <v>36348.2899</v>
+        <v>9914.3861</v>
       </c>
       <c r="I64" s="1" t="s">
         <v>10</v>
@@ -2167,13 +2167,13 @@
         <v>226.1401</v>
       </c>
       <c r="F65" s="1" t="n">
-        <v>1149.6918</v>
+        <v>2310.4489</v>
       </c>
       <c r="G65" s="1" t="n">
-        <v>-22775.3215</v>
+        <v>-5959.8316</v>
       </c>
       <c r="H65" s="1" t="n">
-        <v>23227.6016</v>
+        <v>6412.1117</v>
       </c>
       <c r="I65" s="1" t="s">
         <v>10</v>
@@ -2195,13 +2195,13 @@
         <v>982.5116</v>
       </c>
       <c r="F66" s="1" t="n">
-        <v>1402.1786</v>
+        <v>1148.2663</v>
       </c>
       <c r="G66" s="1" t="n">
-        <v>-27070.3613</v>
+        <v>-2091.8445</v>
       </c>
       <c r="H66" s="1" t="n">
-        <v>29035.3844</v>
+        <v>4056.8676</v>
       </c>
       <c r="I66" s="1" t="s">
         <v>10</v>
@@ -2223,16 +2223,16 @@
         <v>-4302.8166</v>
       </c>
       <c r="F67" s="1" t="n">
-        <v>1918.4202</v>
+        <v>1580.6415</v>
       </c>
       <c r="G67" s="1" t="n">
-        <v>-42683.9446</v>
+        <v>-8534.8096</v>
       </c>
       <c r="H67" s="1" t="n">
-        <v>34078.3113</v>
+        <v>-70.8237</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J67" s="1" t="s">
         <v>13</v>

</xml_diff>